<commit_message>
Add card 22: Shure Wireless Workbench (WWB 6 & 7) compatibility profiles
First software card. Scenario: event coordination assigns exact
frequencies, the crew's WWB rejects them on its own intermod margins
(3TO/spacing warnings). Card walks both WWB 6 and WWB 7 paths to relax
the compatibility profile (Robust/Standard -> More Frequencies), says
explicitly NOT to recalculate new frequencies, and explains the
trade-off. Verified against Shure's current WWB help and the WWB6
compatibility-profiles article.

Builders upgraded for software cards: proc column labels and RF-bar row
labels now flow from print.html into the app segmented control and the
XLSX (no more hardcoded TRANSMITTER/RF POWER labels).
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -29,6 +29,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comtek 216" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sound Devices Astral" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zaxcom" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shure WWB" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -996,29 +997,49 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Shure WWB</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>WWB 6</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>WWB 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>Three rules that prevent most check-in failures</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>1.  Transmitter and receiver must be in the same band / block.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
+          <t>1.  Transmitter and receiver must be in the same band / block.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>3.  On digital systems an IR-sync (RX-&gt;TX) copies the frequency onto the other unit; re-sync after changing encryption or band.</t>
         </is>
@@ -1191,7 +1212,7 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PORTABLE RECEIVER  -  UR4D / UR4S (rack receiver — no portable in-series)</t>
+          <t>RECEIVER (RACK)  -  UR4D / UR4S (rack receiver — no portable in-series)</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1246,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Portable Receiver</t>
+          <t>Receiver (Rack)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1272,7 +1293,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1284,7 +1305,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1621,7 +1642,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1633,7 +1654,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1947,7 +1968,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1959,7 +1980,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2288,7 +2309,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2300,7 +2321,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2644,7 +2665,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2656,7 +2677,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -3000,7 +3021,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -3012,7 +3033,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -3349,7 +3370,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -3361,7 +3382,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -3698,7 +3719,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -3710,7 +3731,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -4062,7 +4083,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4074,7 +4095,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -4419,7 +4440,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4431,7 +4452,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -4791,7 +4812,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -4803,7 +4824,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -5147,7 +5168,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -5159,7 +5180,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -5496,7 +5517,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -5508,7 +5529,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -5860,7 +5881,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -5872,7 +5893,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -5981,6 +6002,378 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Shure Wireless Workbench (WWB 6 &amp; 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Software · making WWB accept coordinator-assigned frequencies · nothing on this card transmits</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>How to reach any MHz</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>SOFTWARE — CALC ONLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Tuning step</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>profiles: Robust · Standard · More Frequencies</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Range / band</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>applies only to the WWB calculator on your laptop — it changes nothing on any transmitter</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Matching TX &lt;-&gt; RX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Deploying from WWB: linked Axient pairs update instantly over ShowLink; UHF-R / ULX-D / PSM1000 update the rack, then IR-sync the portables; everything else is tuned by hand (see that system’s card).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>WWB 6  -  WWB 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Wwb 6</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WWB 6</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Frequency Coordination tab -&gt; click the device-type group header. The header text shows the active profile (“Standard” / “Robust” / “More Frequencies”).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Right sidebar -&gt; Compatibility tab -&gt; Compatibility Profile drop-down -&gt; More Frequencies (try Standard first if you only need a little slack).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Re-enter / keep the assigned freqs and hit [Calculate] — the header text updates and the warnings should clear. (The underlying spacing numbers live in Tools ▸ Equipment Profiles ▸ Filtering &amp; Intermods.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>WWB 7  -  WWB 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Wwb 7</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>WWB 7</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Frequency coordination workspace -&gt; click the device header (dark grey bar); [Ctrl]-click to select several.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Compatibility tab -&gt; profile drop-down -&gt; More frequencies (or Standard). Fine control: Channel spacing / Intermod spacing (2- and 3-transmitter) sliders; [Revert] undoes, [Save] stores a modified profile (shows a *).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Click [Calculate]. Default for every future device: Preferences ▸ Coordination ▸ Compatibility -&gt; double-click the model’s Coordination Preference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>RF POWER &amp; SAFE POWER-ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>DON’T RECALC</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Type the coordinator’s frequencies exactly (double-click the Frequency column in Inventory and type). Relaxing the profile is only to make WWB accept them — don’t press Calculate to generate new frequencies without checking with coordination first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>TRADE-OFF</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>More Frequencies = tighter spacings: less margin against intermod products and short TX-to-RX distances. Fine when the site-wide coordination owns the plan; not a free win when you’re self-coordinating in isolation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>WATCH OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•  “3TO”-style warnings are WWB’s own 2- and 3-transmitter third-order intermod spacing rules — a margin policy, not a verdict on the event plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>•  Set the profile per device type — relax only the types you were handed frequencies for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>•  If WWB still refuses one specific assigned frequency, don’t nudge it to a nearby number — call coordination; the digits are load-bearing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>•  Changing the profile changes calculations only; nothing reaches hardware until you deploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>WWB help — Adjust Compatibility Settings</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>https://content-files.shure.com/Pubs/WWB/en-US/en-US/adjust-compatibility-settings.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>WWB6 compatibility profiles (Shure)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://www.shure.com/en-US/insights/shure-wireless-workbench-6-compatibility-profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>WWB help — Specify a Frequency</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>https://content-files.shure.com/Pubs/WWB/en-US/en-US/specify-a-frequency-for-a-channel.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId3"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6224,7 +6617,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -6236,7 +6629,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -6588,7 +6981,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -6600,7 +6993,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -6929,7 +7322,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -6941,7 +7334,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -7278,7 +7671,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -7290,7 +7683,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -7642,7 +8035,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -7654,7 +8047,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -7991,7 +8384,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -8003,7 +8396,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -8307,7 +8700,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Power on with RF OFF</t>
+          <t>RF OFF FIRST</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -8319,7 +8712,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>RF power</t>
+          <t>RF POWER</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Add Teradek wireless video cards (23-24): channel lock + 5/6 GHz chart
Card 23 - Teradek Bolt / Ranger: lock to one frequency (Menu > Wireless
Settings > Enable Fixed Frequency on BOTH ends + explicitly select the
assigned channel, else Bolt defaults to the lowest in the list) and lock
bandwidth to 20 MHz (Wireless Settings > Bandwidth; 1080p60 max at 20).
Key catch documented: Fixed Frequency offers non-DFS channels only, so
DFS assignments are impossible by design. Ranger licensed-channel note.

Card 24 - 5/6 GHz channel chart: U-NII bands with 20 MHz channel <->
center MHz tables, DFS rows flagged amber, lockable rows green, formula
pills, and the definitive 6 GHz-capable Teradek list (Bolt 6 all SKUs,
Bolt 4K LT-HDMI fw>=4.3.0, Ranger Mk II, Ranger Micro).

All claims verified against guide.teradek.com. Builders: bandtable
support in app+XLSX, brand fallback 'Reference', seg toggle hidden on
cards without TX/RX columns. Deck now 24 cards; PDF 25 pages.
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -30,6 +30,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sound Devices Astral" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zaxcom" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shure WWB" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teradek" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-6 GHz Chart" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +94,11 @@
       <color rgb="FF4A6B86"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -123,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -156,6 +163,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -523,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1017,29 +1027,61 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Teradek</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Same steps on TX and RX</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Same steps on TX and RX</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>5-6 GHz Chart</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Three rules that prevent most check-in failures</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>1.  Transmitter and receiver must be in the same band / block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>1.  Transmitter and receiver must be in the same band / block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>3.  On digital systems an IR-sync (RX-&gt;TX) copies the frequency onto the other unit; re-sync after changing encryption or band.</t>
         </is>
@@ -6362,6 +6404,771 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Teradek Bolt / Ranger (wireless video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>5 / 6 GHz zero-delay video · lock it to one channel so it can’t hop</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>How to reach any MHz</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>LOCK TO ONE CHANNEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Tuning step</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>20 MHz per link (factory default is 40 MHz — twice the footprint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Range / band</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>5 GHz U-NII-1/2/3 · 6 GHz U-NII-5 5.925–6.425 (Bolt 6 · Bolt 4K LT-HDMI · Ranger Mk II/Micro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Matching TX &lt;-&gt; RX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ranger is the special case: spans 4.9–6.0 GHz including licensed channels — enable Allow Licensed Channels + Fixed Frequency to pick one (licensed operations only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>LOCK THE FREQUENCY  -  Same steps on TX and RX</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Lock The Frequency</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Same steps on TX and RX</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>[Menu] -&gt; Wireless Settings -&gt; Enable Fixed Frequency — on both TX and RX (“bypasses any automatic frequency switching logic”).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Then Wireless Settings ▸ Frequencies: select only the assigned channel. If you skip this, Bolt silently defaults to the lowest frequency in the list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Fixed mode offers non-DFS channels only — if your assignment is a DFS channel, the unit cannot lock there; call coordination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>LOCK 20 MHz + BAND  -  Same steps on TX and RX</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Lock 20 Mhz + Band</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Same steps on TX and RX</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>[Menu] -&gt; Wireless Settings -&gt; Bandwidth -&gt; 20MHz (default 40) — both ends must match. 20 MHz carries up to 1080p60; 4K59/60 needs 40 MHz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>6 GHz-capable units: Wireless Settings ▸ Band -&gt; 5GHz or 6GHz per the assignment — both ends; hopping never spans bands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Sanity-check with the Spectrum Analyzer (RX front panel / Bolt app). Changed the Region setting? Re-pair TX and RX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>RF POWER &amp; SAFE POWER-ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>NO DFS LOCK</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Fixed Frequency = non-DFS only. DFS ranges (5.25–5.35 / 5.47–5.725 GHz) need a 1-minute radar scan and can be forced to vacate — don’t assign video links there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>FOOTPRINT</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>6 GHz (U-NII-5) runs at lower allowed power than 5 GHz but has no DFS. At 20 MHz a Bolt 6 offers 36 channel choices vs 24 at 40 MHz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>WATCH OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•  Serv / Prism / Cube are IP encoders on ordinary Wi-Fi — nothing to lock on the unit; coordinate the network instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>•  Frequency, bandwidth, and band must match on both ends or the link won’t form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>•  See the companion 5/6 GHz channel chart card for channel ⇄ MHz mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Bolt 6 wireless configuration</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1601336-wireless-configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Bolt 4K wireless configuration</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1625378-wireless-configuration</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Bolt 6 GHz support by region</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1601470-bolt-6-u-nii-5-6ghz-support-by-region</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Frequencies by region chart</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1589935-frequencies-by-region</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A34:B34"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId4"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>5 / 6 GHz Channel Chart (video &amp; Wi-Fi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generic 20 MHz channelization · channel ⇄ center MHz · who can go to 6 GHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>How to reach any MHz</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>REFERENCE CHART</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Tuning step</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Range / band</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Matching TX &lt;-&gt; RX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>5 GHz band</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Span (MHz)</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>20 MHz channels (center MHz)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>5150–5250</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>36 (5180) · 40 (5200) · 44 (5220) · 48 (5240)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>No DFS — lockable</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-2A</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>5250–5350</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>52 (5260) · 56 (5280) · 60 (5300) · 64 (5320)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>DFS — radar scan, can be evicted</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-2C</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>5470–5725</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>100 (5500) · 104 · 108 · 112 · 116 · 120 · 124 · 128 · 132 · 136 · 140 · 144 (5720)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>DFS — radar scan, can be evicted</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>5725–5850</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>149 (5745) · 153 (5765) · 157 (5785) · 161 (5805) · 165 (5825)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>No DFS — lockable, but shared with venue Wi-Fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>6 GHz band</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Span (MHz)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>20 MHz channels (center MHz)</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-5</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>5925–6425</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>1 (5955) · 5 (5975) · 9 (5995) … step +4 ch / +20 MHz … 93 (6415)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>No DFS; lower power (LPI); only band Teradek uses</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-6</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>6425–6525</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>97 (6435) – 113 (6515)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Wi-Fi 6E/7 only — no Teradek products here; venue APs may be</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>6525–6875</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>117 (6535) – 185 (6875)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>U-NII-8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>6875–7125</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>189 (6895) – 233 (7115)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>RF POWER &amp; SAFE POWER-ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>WATCH OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>•  Teradek fixed-frequency locks only exist in the green rows (U-NII-1, U-NII-3, U-NII-5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>•  A 40 MHz link eats two adjacent 20 MHz slots — count both when charting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•  Venue Wi-Fi lives in these same bands; 6 GHz (U-NII-5) is usually the cleanest room on site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Teradek frequencies by region</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1589935-frequencies-by-region</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Bolt 6 6 GHz support</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>https://guide.teradek.com/a/1601470-bolt-6-u-nii-5-6ghz-support-by-region</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>WLAN channel list (IEEE numbering)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/List_of_WLAN_channels</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="C32:E32"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId3"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Fan Fest report rev 2: extend 4 cards (DCHT, EW-D, TRXCL5, G2)
- D Squared: DCHT camera-hop TX (wideband 470.1-607.950, 25 kHz,
  Xmit > Freq, DCHX mode with DCHR / DSQD fw>=1.04, 10/25/50 mW)
- EW-DX: EW-D sibling notes (TX has no display; freq set on EW-D EM or
  Smart Assist app, pushed via SYNC/BLE; fixed 10 mW; Q1-6 = 470.2-526,
  S1-7 = 606.2-662 mostly non-US) + EW-D manual source link
- Zaxcom: TRXCL5 camera link (same INC/DEC 100 kHz drill; US ranges and
  power tiers) + manual link
- G3/G4: 'EW G2/G3/G4' report label + hedged G2 note

Per coordination policy, no card for auto-hopping 2.4 GHz mics (DJI,
Rode etc.) - not frequency-agile, nothing to coordinate.

All verified against manufacturer docs. No new cards; deck stays 24.
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -4245,7 +4245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4538,74 +4538,97 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>•  DCHT camera-hop TX is family: wideband 470.1–607.950, 25 kHz, Xmit ▸ Freq; pairs with DCHR (native DCHX mode) or DSQD (fw ≥ 1.04); 10 / 25 / 50 mW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>DBSM/DBSMD manual</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>https://lectrosonics.com/wp-content/uploads/filr/1940/DBSM_man_ALL.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>DSQD manual</t>
+          <t>DBSM/DBSMD manual</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>https://lectrosonics.com/wp-content/uploads/filr/3315/DSQDman.pdf</t>
+          <t>https://lectrosonics.com/wp-content/uploads/filr/1940/DBSM_man_ALL.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t>DSQD manual</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>https://lectrosonics.com/wp-content/uploads/filr/3315/DSQDman.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>DSR4 manual</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>https://www.lectrosonics.com/wp-content/uploads/filr/3278/DSR4man.pdf</t>
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>DCHT manual</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>https://lectrosonics.com/wp-content/uploads/filr/3297/DCHT_man_ALL.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="21">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="C33:E33"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A27:E27"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4892,7 +4915,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>•  G3 and G4 tune identically.</t>
+          <t>•  G3 and G4 tune identically. Reports often lump G2 in too — same family drill, but verify menu names on older G2 units at the table.</t>
         </is>
       </c>
     </row>
@@ -5686,7 +5709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -5972,73 +5995,96 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>•  TRXCL5 camera link tunes the same way (INC/DEC, 100 kHz): US 512–607.9 up to 100 mW (+ 614.1–615.9 / 653.1–662.9 at 20 mW); power 25 / 50 / 100 mW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>ZMT4/4.5 manual</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>https://zaxcom.com/wp-content/uploads/2022/01/Zaxcom_ZMT4_Manual_April_2021.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>URX100 manual</t>
+          <t>ZMT4/4.5 manual</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>https://zaxcom.com/wp-content/uploads/2019/05/Zaxcom_URX100_Manual_August_2019.pdf</t>
+          <t>https://zaxcom.com/wp-content/uploads/2022/01/Zaxcom_ZMT4_Manual_April_2021.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>URX100 manual</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://zaxcom.com/wp-content/uploads/2019/05/Zaxcom_URX100_Manual_August_2019.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>VTX1 manual</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>https://zaxcom.com/wp-content/uploads/2025/08/Zaxcom_VTX1_July_2025.pdf</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>TRXCL5 manual</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>https://zaxcom.com/wp-content/uploads/2023/06/Zaxcom_TRXCL5_Manual_August-2022-1.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C35:E35"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7175,7 +7221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7461,73 +7507,96 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>•  EW-D (non-DX) TXs have no display at all — set the freq on the EW-D EM (or Smart Assist app) and push with the [SYNC] buttons (BLE). Fixed 10 mW. Q1-6 = 470.2–526; “S1-7” = 606.2–662 (mostly not US-legal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>EW-D/DX/DP combined manual</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>https://www.sennheiser.com/globalassets/digizuite/40783-en-instruction-manual-and-frequently-asked-questions---evolution-wireless-digital-ew-d--ew-dx--ew-dp-pdf.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>EW-DX online manual</t>
+          <t>EW-D/DX/DP combined manual</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>https://docs.cloud.sennheiser.com/en-us/ew-d/ew-d/manual.html</t>
+          <t>https://www.sennheiser.com/globalassets/digizuite/40783-en-instruction-manual-and-frequently-asked-questions---evolution-wireless-digital-ew-d--ew-dx--ew-dp-pdf.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>EW-DX online manual</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://docs.cloud.sennheiser.com/en-us/ew-d/ew-d/manual.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>Frequency ranges</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>https://docs.cloud.sennheiser.com/en-us/ew-d/ew-d/productinfo-freq-ranges.html</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>EW-D manual</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>https://assets.sennheiser.com/download/assets/ew-d_instruction_manual_06_2026_en.pdf/092d50fcf2f111f0b4c42e4518a8e27d?attachment=true</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C35:E35"/>
     <mergeCell ref="A34:B34"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add card 25: 2.4 GHz auto-hop mics (DJI / Rode / Hollyland)
Explainer card: these cannot be coordinated by design (automatic
frequency hopping, no user channel control on any of the five systems -
verified against DJI, Rode, Hollyland spec pages). Saturation warning:
enough of them clustered in one area fill the shared ISM band and all
start dropping at once. Crew guidance column, FCC Part 15 context, and
a history bonus linking Hedy Lamarr + George Antheil's 1942 FHSS patent
(US 2,292,387). Deck: 25 cards, PDF 26 pages.
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -32,6 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shure WWB" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teradek" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-6 GHz Chart" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.4 GHz Auto-Hop" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1059,29 +1060,49 @@
       <c r="C30" s="5" t="inlineStr"/>
       <c r="D30" s="5" t="inlineStr"/>
     </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>2.4 GHz Auto-Hop</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>All 2.4 GHz ISM, all auto-hop</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Kindly, at the check-in table</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>Three rules that prevent most check-in failures</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>1.  Transmitter and receiver must be in the same band / block.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
+          <t>1.  Transmitter and receiver must be in the same band / block.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>2.  On Sony UWP-D &amp; Wisycom, select the fine / unlocked group before an arbitrary frequency is reachable (Sony DWX also offers direct FREQ INPUT).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>3.  On digital systems an IR-sync (RX-&gt;TX) copies the frequency onto the other unit; re-sync after changing encryption or band.</t>
         </is>
@@ -7215,6 +7236,396 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>2.4 GHz Auto-Hop Mics (DJI / Rode / Hollyland)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Consumer digital mics · adaptive frequency hopping · there is no frequency to dial</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>How to reach any MHz</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>CANNOT BE COORDINATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Tuning step</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>none — the radio picks its own hops, continuously</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Range / band</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2.400–2.4835 GHz ISM (DJI Mic 3 can also use 5.1–5.8 GHz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Matching TX &lt;-&gt; RX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>WHAT THEY ARE  -  All 2.4 GHz ISM, all auto-hop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>What They Are</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>All 2.4 GHz ISM, all auto-hop</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>DJI Mic / Mic 2 / Mic Mini: 2.400–2.4835 GHz, GFSK, &lt; 20 dBm EIRP (Mic 3 adds 5.1–5.8 GHz).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Rode Wireless GO II / PRO / ME: “Series IV” 2.4 GHz digital, 128-bit encryption, auto-pairing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Hollyland Lark M2 / Max: 2.4 GHz adaptive frequency hopping, &lt; 20 dBm EIRP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>WHAT TO TELL THE CREW  -  Kindly, at the check-in table</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Instruction</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Notes / Corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>What To Tell The Crew</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Kindly, at the check-in table</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>These can’t take an assigned frequency — that’s the design, not a setting you’re missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>They share 2.4 GHz with venue Wi-Fi, Bluetooth, ZaxNet, and comms — count them on the walk anyway; every one raises the noise floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Power off units that aren’t actively shooting; if reliability matters, hand them a coordinated UHF pack instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>RF POWER &amp; SAFE POWER-ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>SATURATION</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Saturation is the endgame: each link needs clean hop-space. Cluster enough of them (plus Wi-Fi, Bluetooth, ZaxNet) in one small area and the band fills — all of them start dropping at once, and no settings menu can fix physics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>RF POWER</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Fixed by regulation, not by menu: ISM-band devices run &lt; 20 dBm EIRP and must tolerate each other’s interference (FCC Part 15). Range claims (100–400 m LOS) assume a quiet band — an event floor is not one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>WATCH OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•  Nothing on this card is field-tunable — if a crew insists their unit “has a channel setting,” it’s a pairing menu, not a frequency menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>•  DJI Mic 3 in 5 GHz mode lands in the same U-NII bands as Teradek video — see the 5/6 GHz chart card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>•  These are fine tools in isolation; the problem is density.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>SOURCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>DJI Mic 2 specs</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>https://www.dji.com/mic-2/specs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Rode Wireless GO II</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>https://rode.com/en-us/microphones/wireless/wirelessgoii</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Hollyland Lark Max specs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>https://www.hollyland.com/product/lark-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Lamarr FHSS patent (1942)</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>https://patents.google.com/patent/US2292387A/en</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Hedy Lamarr — MIT Lemelson</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>https://lemelson.mit.edu/resources/hedy-lamarr</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="A34:B34"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Sony DWX: GP 00 is the free-tune path on DWT transmitters
Per coordinator practice, confirmed against Sony's DWX frequency list:
Group 00 spans the unit's whole band in 125 kHz steps ('permits the
units to operate on any... carrier frequencies in 125-kHz steps';
Sony notes simultaneous multi-channel operation is not assured - i.e.
not intermod-protected, which is fine under external coordination).
TX step 2 now says pick GP 00 for free tuning; TV-channel groups remain
the 25 kHz path for .025/.075 offsets; caveat added.
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>[+]/[–] to GP/CH; hold [SET] until GROUP flashes -&gt; pick the TV-channel group; [SET].</t>
+          <t>[+]/[–] to GP/CH; hold [SET] until GROUP flashes -&gt; pick GP 00 for free tuning (any freq on the 125 kHz raster); [SET].</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>CHANNEL flashes -&gt; set to the channel = assigned MHz; [SET]. Power-cycle to transmit.</t>
+          <t>CHANNEL flashes -&gt; set to the channel = assigned MHz; [SET]. Power-cycle to transmit. (Assignment on a .025/.075 offset? GP 00 can’t land there — use the TV-channel group instead.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lectrosonics cards: exact RF-power-setting procedures on the TX side
Verified against Lectrosonics manuals:
- SMV/SMQV: set from OFF via hold UP + AUDIO+FREQ hidden setup mode,
  step to the Pr screen (same mode as compat setup - explains the old
  standby-boot mixup); 941 variants capped at 50/100
- LT: MENU/SEL > TxPower (50/100); SMWB/SMDWB same path but 25/50/100;
  LMb fixed 50 mW, no menu
- IFBT2.0: RF ENABLE/LEVEL per carrier (10-250 mW) + must exit setup
  screen before power-down; IFBT4 fixed ~250 mW
- M2T Duet: RF ENABLE/LEVEL button sequence per carrier
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -3101,7 +3101,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>50 / 100 / 250 mW in the Power menu (250 mW not on the 941 band).</t>
+          <t>50 / 100 / 250 mW (941 variants: 50/100). Set from OFF: hold [UP], press [AUDIO]+[FREQ] together -&gt; step to the Pr screen ([AUDIO]/[FREQ]) -&gt; [▲▼] to pick -&gt; [AUDIO]+[FREQ] to exit, then power on.</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>50 / 100 mW (Power menu).</t>
+          <t>LT: [MENU/SEL] -&gt; TxPower -&gt; [▲▼] 50 / 100 mW -&gt; [MENU/SEL]. SMWB/SMDWB, same path: 25 / 50 / 100 mW. LMb: fixed 50 mW — no menu.</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>IFBT4: ~250 mW. IFBT2.0: selectable 10 / 25 / 50 / 100 / 250 mW.</t>
+          <t>IFBT4: fixed ≈250 mW. IFBT2.0: [MENU/SEL] -&gt; RF ENABLE/LEVEL -&gt; [SEL] per carrier -&gt; [▲▼] 10 / 25 / 50 / 100 / 250 mW; leave the setup screen before power-down or it won’t save.</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>10 / 25 / 50 mW per carrier (RF Enable/Level menu).</t>
+          <t>[MENU/SEL] -&gt; RF ENABLE/LEVEL -&gt; [SEL] steps carrier/field -&gt; [▲▼] to enable and set 10 / 25 / 50 mW per carrier -&gt; [BACK].</t>
         </is>
       </c>
     </row>

</xml_diff>